<commit_message>
Support composite family map keys
</commit_message>
<xml_diff>
--- a/Backend/data/family_map.xlsx
+++ b/Backend/data/family_map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a30aadf1b7f22e9a/Cartella progetto/product-finder 2/Backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="220" documentId="8_{9F845F45-37D4-46D6-A0A5-681E85BF7A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D699182-E1E8-44EF-B737-E29455B1F2F2}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="8_{9F845F45-37D4-46D6-A0A5-681E85BF7A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6EAD354-2703-4E64-84EC-852C2C506FFC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{33666627-96C5-49B9-9BBD-E8D72ECEEC80}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1345" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="651">
   <si>
     <t>Waterproof</t>
   </si>
@@ -1988,6 +1988,9 @@
   </si>
   <si>
     <t>highbay</t>
+  </si>
+  <si>
+    <t>Roda</t>
   </si>
 </sst>
 </file>
@@ -2062,8 +2065,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DEA0505-44D9-4A4C-91A0-3353BBB1D1C9}" name="Tabella1" displayName="Tabella1" ref="A1:C667" totalsRowShown="0">
-  <autoFilter ref="A1:C667" xr:uid="{8DEA0505-44D9-4A4C-91A0-3353BBB1D1C9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DEA0505-44D9-4A4C-91A0-3353BBB1D1C9}" name="Tabella1" displayName="Tabella1" ref="A1:C668" totalsRowShown="0">
+  <autoFilter ref="A1:C668" xr:uid="{8DEA0505-44D9-4A4C-91A0-3353BBB1D1C9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C667">
     <sortCondition sortBy="cellColor" ref="C1:C6439" dxfId="1"/>
   </sortState>
@@ -2393,10 +2396,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C7A7BAF-2E6C-4A12-BE1C-DDCF5E136ECB}">
-  <dimension ref="A1:K667"/>
+  <dimension ref="A1:K668"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="85.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -9852,8 +9856,19 @@
         <v>Vertical</v>
       </c>
     </row>
+    <row r="668" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A668" t="s">
+        <v>650</v>
+      </c>
+      <c r="B668" t="s">
+        <v>0</v>
+      </c>
+      <c r="C668">
+        <v>1782</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C667">
+  <conditionalFormatting sqref="C2:C668">
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>